<commit_message>
docs: 정합 정리 — xlsx IA 최신화 · design.md §5 Auth 분리 · 25MB html 제거
- 화면정의서 xlsx(SSOT+frontend): SCR-021 핫딜 전용·지마켓 삭제, 홈/장바구니 시세추천 (PR#22 닫히며 유실됐던 IA 수정 복원)
- design.md §5: User/Auth 분리 반영 (7→8 서비스), §10 확정 표시
- docs/design/food-budget 공유용.html(25MB) 제거 — 로컬 확정본이 최신, 렌더 번들은 gitignore(로컬만)

Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/design/frontend specification.xlsx
+++ b/docs/design/frontend specification.xlsx
@@ -132,7 +132,7 @@
     <x:t xml:space="preserve">홈 대시보드</x:t>
   </x:si>
   <x:si>
-    <x:t xml:space="preserve">예산·재고·추천·성과·최근 지출 요약</x:t>
+    <x:t xml:space="preserve">예산·재고·추천·성과·최근 지출·지금 싼 재료(시세추천) 요약</x:t>
   </x:si>
   <x:si>
     <x:t xml:space="preserve">로그인/예산 설정 완료</x:t>
@@ -285,7 +285,7 @@
     <x:t xml:space="preserve">장바구니</x:t>
   </x:si>
   <x:si>
-    <x:t xml:space="preserve">부족 재료 합산·가격·예산 비교</x:t>
+    <x:t xml:space="preserve">부족 재료 합산·가격·예산 비교·지금 싼 재료 추천</x:t>
   </x:si>
   <x:si>
     <x:t xml:space="preserve">추천에서 장보기 목록 만들기 / 전역 장바구니</x:t>
@@ -444,10 +444,10 @@
     <x:t xml:space="preserve">가격</x:t>
   </x:si>
   <x:si>
-    <x:t xml:space="preserve">핫딜·시세</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">저렴한 재료·할인율·관련 레시피 제공</x:t>
+    <x:t xml:space="preserve">핫딜</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">오아시스 타임/마감세일·할인율·관련 레시피 제공</x:t>
   </x:si>
   <x:si>
     <x:t xml:space="preserve">홈 뭐 사지 / P1 메뉴</x:t>
@@ -456,7 +456,7 @@
     <x:t xml:space="preserve">장바구니 추가 또는 외부 상품 이동</x:t>
   </x:si>
   <x:si>
-    <x:t xml:space="preserve">지마켓 타임딜 포함</x:t>
+    <x:t xml:space="preserve">오아시스 타임세일(15시)·마감세일(17시) / 시세추천은 홈·장바구니 임베드</x:t>
   </x:si>
   <x:si>
     <x:t xml:space="preserve">SCR-022</x:t>

</xml_diff>

<commit_message>
chore(frontend): frontend 스캐폴드 — 화면정의서·아이콘 + 대용량 html gitignore (#30)
* chore(frontend): frontend 스캐폴드 — 화면정의서·앱 아이콘 + 대용량 html gitignore

- frontend/references/: 프론트엔드 화면정의서.pdf, 화면정의서.xlsx (개발 기준)
- frontend/public/icons/app-icon.png: 앱 메인 + 챗봇 아이콘 공용
- frontend/README.md: 개발 기준·스택·화면(SCR-001~022) 안내
- .gitignore: 밀플래닝 확정본.html(25MB)·food-budget 공유용.html·Zone.Identifier·db-connection-guide/.env/.pgpass

Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>

* docs: 정합 정리 — xlsx IA 최신화 · design.md §5 Auth 분리 · 25MB html 제거

- 화면정의서 xlsx(SSOT+frontend): SCR-021 핫딜 전용·지마켓 삭제, 홈/장바구니 시세추천 (PR#22 닫히며 유실됐던 IA 수정 복원)
- design.md §5: User/Auth 분리 반영 (7→8 서비스), §10 확정 표시
- docs/design/food-budget 공유용.html(25MB) 제거 — 로컬 확정본이 최신, 렌더 번들은 gitignore(로컬만)

Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>

---------

Co-authored-by: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/design/frontend specification.xlsx
+++ b/docs/design/frontend specification.xlsx
@@ -132,7 +132,7 @@
     <x:t xml:space="preserve">홈 대시보드</x:t>
   </x:si>
   <x:si>
-    <x:t xml:space="preserve">예산·재고·추천·성과·최근 지출 요약</x:t>
+    <x:t xml:space="preserve">예산·재고·추천·성과·최근 지출·지금 싼 재료(시세추천) 요약</x:t>
   </x:si>
   <x:si>
     <x:t xml:space="preserve">로그인/예산 설정 완료</x:t>
@@ -285,7 +285,7 @@
     <x:t xml:space="preserve">장바구니</x:t>
   </x:si>
   <x:si>
-    <x:t xml:space="preserve">부족 재료 합산·가격·예산 비교</x:t>
+    <x:t xml:space="preserve">부족 재료 합산·가격·예산 비교·지금 싼 재료 추천</x:t>
   </x:si>
   <x:si>
     <x:t xml:space="preserve">추천에서 장보기 목록 만들기 / 전역 장바구니</x:t>
@@ -444,10 +444,10 @@
     <x:t xml:space="preserve">가격</x:t>
   </x:si>
   <x:si>
-    <x:t xml:space="preserve">핫딜·시세</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">저렴한 재료·할인율·관련 레시피 제공</x:t>
+    <x:t xml:space="preserve">핫딜</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">오아시스 타임/마감세일·할인율·관련 레시피 제공</x:t>
   </x:si>
   <x:si>
     <x:t xml:space="preserve">홈 뭐 사지 / P1 메뉴</x:t>
@@ -456,7 +456,7 @@
     <x:t xml:space="preserve">장바구니 추가 또는 외부 상품 이동</x:t>
   </x:si>
   <x:si>
-    <x:t xml:space="preserve">지마켓 타임딜 포함</x:t>
+    <x:t xml:space="preserve">오아시스 타임세일(15시)·마감세일(17시) / 시세추천은 홈·장바구니 임베드</x:t>
   </x:si>
   <x:si>
     <x:t xml:space="preserve">SCR-022</x:t>

</xml_diff>